<commit_message>
feat task member permission
</commit_message>
<xml_diff>
--- a/src/styles/task/Task Event Template.xlsx
+++ b/src/styles/task/Task Event Template.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>Title</t>
   </si>
@@ -51,37 +51,267 @@
     <t>Description</t>
   </si>
   <si>
+    <t>Color</t>
+  </si>
+  <si>
     <t>Repeat Type</t>
   </si>
   <si>
     <t>None</t>
   </si>
   <si>
+    <t>Blue</t>
+  </si>
+  <si>
     <t>Daily</t>
   </si>
   <si>
+    <t>Red</t>
+  </si>
+  <si>
     <t>Weekly</t>
   </si>
   <si>
+    <t>Yellow</t>
+  </si>
+  <si>
     <t>Monthly</t>
   </si>
   <si>
+    <t>Green</t>
+  </si>
+  <si>
     <t>Yearly</t>
   </si>
   <si>
-    <t>Required: title; event_title is optional to override event title (backward compatible)</t>
-  </si>
-  <si>
-    <t>Optional: all_day, repeat_* fields, location, guests (comma-separated), description, color</t>
-  </si>
-  <si>
-    <t>repeat_type: none/daily/weekly/monthly/yearly/weekday/custom</t>
-  </si>
-  <si>
-    <t>Dates: dd/mm/yyyy; Times: hh:mm; leave times empty if all_day is true</t>
-  </si>
-  <si>
-    <t>Each row creates a task and an event if event fields are present</t>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>Pink</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Cyan</t>
+  </si>
+  <si>
+    <t>Indigo</t>
+  </si>
+  <si>
+    <t>Gray</t>
+  </si>
+  <si>
+    <t>Slate</t>
+  </si>
+  <si>
+    <t>Stone</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Zinc</t>
+  </si>
+  <si>
+    <t>Rose</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>Lime</t>
+  </si>
+  <si>
+    <t>Emerald</t>
+  </si>
+  <si>
+    <t>Teal</t>
+  </si>
+  <si>
+    <t>Sky</t>
+  </si>
+  <si>
+    <t>Violet</t>
+  </si>
+  <si>
+    <t>Fuchsia</t>
+  </si>
+  <si>
+    <r>
+      <t>Title:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The name or title of the task/event (required).
+Optional Fields
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Start Date:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start date of the task/event. Format: dd/mm/yyyy
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Start Time:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start time in hh:mm format. Leave empty for all-day events.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>End Time:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The end time in hh:mm format. Leave empty if not applicable.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Repeat:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Defines how often the event repeats.
+Valid values:
+None — No repetition
+Daily — Repeats every day
+Weekly — Repeats every week
+Monthly — Repeats every month
+Yearly — Repeats every year
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>To Date:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The end date for the repeating event (if applicable). Format: dd/mm/yyyy
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Description:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Additional notes or details about the task/event.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Color:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Select a display color for the event.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -94,7 +324,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -103,8 +333,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="12"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -276,6 +520,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -313,12 +563,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -570,28 +814,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -600,128 +835,151 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1105,8 +1363,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelRow="7"/>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="5.08333333333333" customWidth="1"/>
     <col min="2" max="2" width="9.66666666666667" customWidth="1"/>
@@ -1115,66 +1373,186 @@
     <col min="5" max="5" width="7.25" customWidth="1"/>
     <col min="6" max="6" width="7.83333333333333" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="5.83333333333333" customWidth="1"/>
     <col min="10" max="10" width="11.9166666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="2:6">
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="10:10">
-      <c r="J3" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="10:10">
-      <c r="J4" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="10:10">
-      <c r="J5" s="5" t="s">
+      <c r="K1" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11">
+      <c r="B2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="F2" s="4"/>
+      <c r="J2" s="7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="10:10">
-      <c r="J6" s="5" t="s">
+      <c r="K2" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="10:10">
-      <c r="J7" s="5" t="s">
+    <row r="3" spans="10:11">
+      <c r="J3" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="10:10">
-      <c r="J8" s="5" t="s">
+      <c r="K3" s="9" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="10:11">
+      <c r="J4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="10:11">
+      <c r="J5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="10:11">
+      <c r="J6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="10:11">
+      <c r="J7" s="10"/>
+      <c r="K7" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="10:11">
+      <c r="J8" s="10"/>
+      <c r="K8" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="10:11">
+      <c r="J9" s="10"/>
+      <c r="K9" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="10:11">
+      <c r="J10" s="10"/>
+      <c r="K10" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="10:11">
+      <c r="J11" s="10"/>
+      <c r="K11" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="10:11">
+      <c r="J12" s="10"/>
+      <c r="K12" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="10:11">
+      <c r="J13" s="10"/>
+      <c r="K13" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="10:11">
+      <c r="J14" s="10"/>
+      <c r="K14" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="10:11">
+      <c r="J15" s="10"/>
+      <c r="K15" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="10:11">
+      <c r="J16" s="10"/>
+      <c r="K16" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="10:11">
+      <c r="J17" s="10"/>
+      <c r="K17" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="10:11">
+      <c r="J18" s="10"/>
+      <c r="K18" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="10:11">
+      <c r="J19" s="10"/>
+      <c r="K19" s="11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="10:11">
+      <c r="J20" s="10"/>
+      <c r="K20" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="10:11">
+      <c r="J21" s="10"/>
+      <c r="K21" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="10:11">
+      <c r="J22" s="10"/>
+      <c r="K22" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="10:11">
+      <c r="J23" s="10"/>
+      <c r="K23" s="11" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1191,42 +1569,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelRow="4"/>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="81.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
+    <row r="1" ht="232.5" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:A2 A4:A5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: membership workspace task
</commit_message>
<xml_diff>
--- a/src/styles/task/Task Event Template.xlsx
+++ b/src/styles/task/Task Event Template.xlsx
@@ -54,91 +54,15 @@
     <t>Color</t>
   </si>
   <si>
-    <t>Repeat Type</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>Yellow</t>
-  </si>
-  <si>
-    <t>Monthly</t>
-  </si>
-  <si>
-    <t>Green</t>
-  </si>
-  <si>
-    <t>Yearly</t>
-  </si>
-  <si>
-    <t>Purple</t>
-  </si>
-  <si>
-    <t>Pink</t>
-  </si>
-  <si>
-    <t>Orange</t>
-  </si>
-  <si>
-    <t>Cyan</t>
-  </si>
-  <si>
-    <t>Indigo</t>
-  </si>
-  <si>
-    <t>Gray</t>
-  </si>
-  <si>
-    <t>Slate</t>
-  </si>
-  <si>
-    <t>Stone</t>
-  </si>
-  <si>
-    <t>Neutral</t>
-  </si>
-  <si>
-    <t>Zinc</t>
-  </si>
-  <si>
-    <t>Rose</t>
-  </si>
-  <si>
-    <t>Amber</t>
-  </si>
-  <si>
-    <t>Lime</t>
-  </si>
-  <si>
-    <t>Emerald</t>
-  </si>
-  <si>
-    <t>Teal</t>
-  </si>
-  <si>
-    <t>Sky</t>
-  </si>
-  <si>
-    <t>Violet</t>
-  </si>
-  <si>
-    <t>Fuchsia</t>
-  </si>
-  <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Title:</t>
     </r>
     <r>
@@ -313,6 +237,90 @@
       <t xml:space="preserve"> Select a display color for the event.</t>
     </r>
   </si>
+  <si>
+    <t>Repeat Type</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>Yellow</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>Yearly</t>
+  </si>
+  <si>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>Pink</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Cyan</t>
+  </si>
+  <si>
+    <t>Indigo</t>
+  </si>
+  <si>
+    <t>Gray</t>
+  </si>
+  <si>
+    <t>Slate</t>
+  </si>
+  <si>
+    <t>Stone</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Zinc</t>
+  </si>
+  <si>
+    <t>Rose</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>Lime</t>
+  </si>
+  <si>
+    <t>Emerald</t>
+  </si>
+  <si>
+    <t>Teal</t>
+  </si>
+  <si>
+    <t>Sky</t>
+  </si>
+  <si>
+    <t>Violet</t>
+  </si>
+  <si>
+    <t>Fuchsia</t>
+  </si>
 </sst>
 </file>
 
@@ -514,13 +522,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -886,7 +894,7 @@
     <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -959,27 +967,29 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1378,187 +1388,135 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>7</v>
-      </c>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
     </row>
     <row r="2" spans="2:11">
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="F2" s="4"/>
-      <c r="J2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="10:11">
-      <c r="J3" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="10:11">
-      <c r="J4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="10"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="5:11">
+      <c r="E3" s="12"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="5:11">
+      <c r="E4" s="12"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="5"/>
     </row>
     <row r="5" spans="10:11">
-      <c r="J5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>16</v>
-      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="5"/>
     </row>
     <row r="6" spans="10:11">
-      <c r="J6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>18</v>
-      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="5"/>
     </row>
     <row r="7" spans="10:11">
-      <c r="J7" s="10"/>
-      <c r="K7" s="9" t="s">
-        <v>19</v>
-      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="5"/>
     </row>
     <row r="8" spans="10:11">
-      <c r="J8" s="10"/>
-      <c r="K8" s="11" t="s">
-        <v>20</v>
-      </c>
+      <c r="J8" s="7"/>
+      <c r="K8" s="8"/>
     </row>
     <row r="9" spans="10:11">
-      <c r="J9" s="10"/>
-      <c r="K9" s="11" t="s">
-        <v>21</v>
-      </c>
+      <c r="J9" s="7"/>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="10:11">
-      <c r="J10" s="10"/>
-      <c r="K10" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="J10" s="7"/>
+      <c r="K10" s="8"/>
     </row>
     <row r="11" spans="10:11">
-      <c r="J11" s="10"/>
-      <c r="K11" s="11" t="s">
-        <v>23</v>
-      </c>
+      <c r="J11" s="7"/>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="10:11">
-      <c r="J12" s="10"/>
-      <c r="K12" s="11" t="s">
-        <v>24</v>
-      </c>
+      <c r="J12" s="7"/>
+      <c r="K12" s="8"/>
     </row>
     <row r="13" spans="10:11">
-      <c r="J13" s="10"/>
-      <c r="K13" s="11" t="s">
-        <v>25</v>
-      </c>
+      <c r="J13" s="7"/>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="10:11">
-      <c r="J14" s="10"/>
-      <c r="K14" s="11" t="s">
-        <v>26</v>
-      </c>
+      <c r="J14" s="7"/>
+      <c r="K14" s="8"/>
     </row>
     <row r="15" spans="10:11">
-      <c r="J15" s="10"/>
-      <c r="K15" s="11" t="s">
-        <v>27</v>
-      </c>
+      <c r="J15" s="7"/>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="10:11">
-      <c r="J16" s="10"/>
-      <c r="K16" s="11" t="s">
-        <v>28</v>
-      </c>
+      <c r="J16" s="7"/>
+      <c r="K16" s="8"/>
     </row>
     <row r="17" spans="10:11">
-      <c r="J17" s="10"/>
-      <c r="K17" s="11" t="s">
-        <v>29</v>
-      </c>
+      <c r="J17" s="7"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" spans="10:11">
-      <c r="J18" s="10"/>
-      <c r="K18" s="11" t="s">
-        <v>30</v>
-      </c>
+      <c r="J18" s="7"/>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" spans="10:11">
-      <c r="J19" s="10"/>
-      <c r="K19" s="11" t="s">
-        <v>31</v>
-      </c>
+      <c r="J19" s="7"/>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" spans="10:11">
-      <c r="J20" s="10"/>
-      <c r="K20" s="11" t="s">
-        <v>32</v>
-      </c>
+      <c r="J20" s="7"/>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" spans="10:11">
-      <c r="J21" s="10"/>
-      <c r="K21" s="11" t="s">
-        <v>33</v>
-      </c>
+      <c r="J21" s="7"/>
+      <c r="K21" s="8"/>
     </row>
     <row r="22" spans="10:11">
-      <c r="J22" s="10"/>
-      <c r="K22" s="11" t="s">
-        <v>34</v>
-      </c>
+      <c r="J22" s="7"/>
+      <c r="K22" s="8"/>
     </row>
     <row r="23" spans="10:11">
-      <c r="J23" s="10"/>
-      <c r="K23" s="11" t="s">
-        <v>35</v>
-      </c>
+      <c r="J23" s="7"/>
+      <c r="K23" s="8"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E$1:E$1048576">
-      <formula1>$J$4:$J$8</formula1>
+      <formula1>Instructions!$B$3:$B$7</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H$1:H$1048576">
+      <formula1>Instructions!$C$3:$C$24</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1569,21 +1527,175 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelRow="5"/>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="81.75" customWidth="1"/>
+    <col min="2" max="2" width="11.9166666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="232.5" spans="1:1">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="2:3">
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" s="7"/>
+      <c r="C8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3">
+      <c r="B9" s="7"/>
+      <c r="C9" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3">
+      <c r="B10" s="7"/>
+      <c r="C10" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3">
+      <c r="B11" s="7"/>
+      <c r="C11" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3">
+      <c r="B12" s="7"/>
+      <c r="C12" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3">
+      <c r="B13" s="7"/>
+      <c r="C13" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3">
+      <c r="B14" s="7"/>
+      <c r="C14" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3">
+      <c r="B15" s="7"/>
+      <c r="C15" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3">
+      <c r="B16" s="7"/>
+      <c r="C16" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="7"/>
+      <c r="C17" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="7"/>
+      <c r="C18" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="7"/>
+      <c r="C19" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="7"/>
+      <c r="C20" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" s="7"/>
+      <c r="C21" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="7"/>
+      <c r="C22" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" s="7"/>
+      <c r="C23" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="7"/>
+      <c r="C24" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="2"/>
-    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B7">
+      <formula1>$B$3:$B$7</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>